<commit_message>
SSD1963 color fix, board-switching via ProjectConfig.h, README update
- Fix SSD1963 parallel color byte-swap: pushBlock and pushPixels no longer
  do RGB565->18-bit conversion for SSD1963; pushColor uses tft_Write_16N
  (no swap) for non-RA8876 drivers so PIO sends MSB first natively
- Introduce ProjectConfig.h as single source of truth for board/driver
  selection; BoardSettings.h includes it so all translation units agree
- Add DISPLAY_DRIVER_RA8876_NATIVE option to ProjectConfig.h for v2.7
- Update README Board Selection and Display Driver sections to reflect
  two-file switch procedure (ProjectConfig.h + User_Setup_LCC_Active.h)
- Add TFT_eSPI_LCC_Setup.h bridge file (documents sketch-side intent)
- Update DisplayConfig_SSD1963_parallel.h: SSD1963_800BD_DRIVER, TOUCH_CS -1
- Minor DisplayDriver.cpp and UserInterface tweaks for v2.7 native mode

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/rp-pico-2-pin-planner-LCCboards.xlsx
+++ b/Documentation/rp-pico-2-pin-planner-LCCboards.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Attic\Documents\Sandboxing\LCC_RPiPico_Turntable\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F680200-235D-4E61-B98C-32A39AE31F59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597FE2EC-6856-4D16-AE35-25CD9EA5C488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8475" yWindow="285" windowWidth="40470" windowHeight="15345" activeTab="1" xr2:uid="{9994E188-9327-AB46-AF3F-8738237FB097}"/>
+    <workbookView xWindow="8475" yWindow="0" windowWidth="40470" windowHeight="20985" xr2:uid="{9994E188-9327-AB46-AF3F-8738237FB097}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="157">
   <si>
     <t>gp0</t>
   </si>
@@ -400,18 +400,6 @@
     <t>I/0-2:Pin4 : SPI1 SDO</t>
   </si>
   <si>
-    <t>I/0-2:Pin7 : open</t>
-  </si>
-  <si>
-    <t>I/0-2:Pin8 : Touch INT</t>
-  </si>
-  <si>
-    <t>I/0-2:Pin9 : Touch I2C0 SDA</t>
-  </si>
-  <si>
-    <t>I/0-2:Pin10 : Touch I2C0 SCL</t>
-  </si>
-  <si>
     <t>LCC Rpi Pico Shield</t>
   </si>
   <si>
@@ -502,7 +490,13 @@
     <t>I/0-2:Pin10 : open</t>
   </si>
   <si>
-    <t>I/0-2:Pin8 : Display Reset</t>
+    <t>I/0-2:Pin9 : Touch INT</t>
+  </si>
+  <si>
+    <t>I/0-2:Pin9 : Display Reset</t>
+  </si>
+  <si>
+    <t>TT-Pin1 - open</t>
   </si>
 </sst>
 </file>
@@ -804,7 +798,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -934,6 +928,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1280,13 +1277,13 @@
   <dimension ref="A1:M54"/>
   <sheetFormatPr defaultColWidth="11.08984375" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="5.81640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.54296875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.7265625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="2.81640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.26953125" customWidth="1"/>
+    <col min="7" max="7" width="20.26953125" hidden="1" customWidth="1"/>
     <col min="8" max="10" width="20.26953125" style="1" customWidth="1"/>
     <col min="11" max="11" width="20.26953125" customWidth="1"/>
     <col min="12" max="12" width="24.26953125" customWidth="1"/>
@@ -1298,19 +1295,22 @@
         <v>58</v>
       </c>
       <c r="B1" s="44" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C1" s="44"/>
       <c r="D1" s="44"/>
       <c r="E1" s="45"/>
-      <c r="G1" t="s">
-        <v>59</v>
-      </c>
-      <c r="H1" s="31">
-        <v>46101</v>
-      </c>
       <c r="I1" s="31"/>
       <c r="J1" s="31"/>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="46">
+        <v>46137</v>
+      </c>
+      <c r="D2" s="46"/>
     </row>
     <row r="3" spans="1:13" ht="18.75" thickBot="1">
       <c r="B3" s="1">
@@ -1354,16 +1354,16 @@
     </row>
     <row r="8" spans="1:13" ht="18.75" thickBot="1">
       <c r="G8" s="30" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H8" s="30" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="I8" s="30" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="J8" s="30" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="K8" s="30" t="s">
         <v>94</v>
@@ -1372,7 +1372,7 @@
         <v>93</v>
       </c>
       <c r="M8" s="30" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1397,7 +1397,9 @@
       <c r="H9" t="s">
         <v>78</v>
       </c>
-      <c r="I9"/>
+      <c r="I9" s="43" t="s">
+        <v>119</v>
+      </c>
       <c r="J9" s="43" t="s">
         <v>119</v>
       </c>
@@ -1405,7 +1407,7 @@
         <v>95</v>
       </c>
       <c r="L9" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="M9" t="s">
         <v>86</v>
@@ -1433,7 +1435,9 @@
       <c r="H10" t="s">
         <v>79</v>
       </c>
-      <c r="I10"/>
+      <c r="I10" s="43" t="s">
+        <v>119</v>
+      </c>
       <c r="J10" s="43" t="s">
         <v>119</v>
       </c>
@@ -1441,7 +1445,7 @@
         <v>96</v>
       </c>
       <c r="L10" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="M10" t="s">
         <v>87</v>
@@ -1480,9 +1484,11 @@
       <c r="H12" t="s">
         <v>80</v>
       </c>
-      <c r="I12"/>
+      <c r="I12" t="s">
+        <v>130</v>
+      </c>
       <c r="J12" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="K12" s="42" t="s">
         <v>97</v>
@@ -1514,15 +1520,17 @@
       <c r="H13" t="s">
         <v>63</v>
       </c>
-      <c r="I13"/>
+      <c r="I13" t="s">
+        <v>131</v>
+      </c>
       <c r="J13" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="K13" s="42" t="s">
         <v>98</v>
       </c>
       <c r="L13" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="M13" s="38" t="s">
         <v>89</v>
@@ -1550,7 +1558,9 @@
       <c r="H14" t="s">
         <v>64</v>
       </c>
-      <c r="I14"/>
+      <c r="I14" s="1" t="s">
+        <v>42</v>
+      </c>
       <c r="J14" s="1" t="s">
         <v>42</v>
       </c>
@@ -1586,7 +1596,9 @@
       <c r="H15" t="s">
         <v>65</v>
       </c>
-      <c r="I15"/>
+      <c r="I15" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="J15" s="1" t="s">
         <v>43</v>
       </c>
@@ -1633,9 +1645,11 @@
       <c r="H17" t="s">
         <v>73</v>
       </c>
-      <c r="I17"/>
+      <c r="I17" t="s">
+        <v>132</v>
+      </c>
       <c r="J17" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="K17" s="42" t="s">
         <v>101</v>
@@ -1667,9 +1681,11 @@
       <c r="H18" t="s">
         <v>66</v>
       </c>
-      <c r="I18"/>
+      <c r="I18" t="s">
+        <v>133</v>
+      </c>
       <c r="J18" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="K18" s="42" t="s">
         <v>102</v>
@@ -1703,9 +1719,11 @@
       <c r="H19" t="s">
         <v>67</v>
       </c>
-      <c r="I19"/>
+      <c r="I19" s="42" t="s">
+        <v>102</v>
+      </c>
       <c r="J19" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="K19" s="42" t="s">
         <v>103</v>
@@ -1739,9 +1757,11 @@
       <c r="H20" t="s">
         <v>68</v>
       </c>
-      <c r="I20"/>
+      <c r="I20" s="42" t="s">
+        <v>101</v>
+      </c>
       <c r="J20" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="K20" s="42" t="s">
         <v>104</v>
@@ -1762,7 +1782,7 @@
       </c>
       <c r="E21" s="20"/>
       <c r="H21"/>
-      <c r="I21"/>
+      <c r="I21" s="42"/>
       <c r="K21" s="42"/>
       <c r="M21" s="42"/>
     </row>
@@ -1786,9 +1806,11 @@
       <c r="H22" t="s">
         <v>69</v>
       </c>
-      <c r="I22"/>
+      <c r="I22" s="42" t="s">
+        <v>146</v>
+      </c>
       <c r="J22" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="K22" s="42" t="s">
         <v>105</v>
@@ -1820,9 +1842,11 @@
       <c r="H23" t="s">
         <v>70</v>
       </c>
-      <c r="I23"/>
+      <c r="I23" s="42" t="s">
+        <v>145</v>
+      </c>
       <c r="J23" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="K23" s="42" t="s">
         <v>106</v>
@@ -1856,18 +1880,20 @@
       <c r="H24" t="s">
         <v>71</v>
       </c>
-      <c r="I24"/>
+      <c r="I24" s="42" t="s">
+        <v>98</v>
+      </c>
       <c r="J24" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="K24" s="42" t="s">
         <v>109</v>
       </c>
-      <c r="L24" s="42" t="s">
-        <v>124</v>
+      <c r="L24" t="s">
+        <v>151</v>
       </c>
       <c r="M24" s="42" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -1892,18 +1918,20 @@
       <c r="H25" t="s">
         <v>72</v>
       </c>
-      <c r="I25"/>
+      <c r="I25" s="42" t="s">
+        <v>97</v>
+      </c>
       <c r="J25" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="K25" s="42" t="s">
         <v>112</v>
       </c>
       <c r="L25" t="s">
-        <v>125</v>
+        <v>152</v>
       </c>
       <c r="M25" s="42" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -1915,7 +1943,7 @@
       </c>
       <c r="E26" s="20"/>
       <c r="H26"/>
-      <c r="I26"/>
+      <c r="I26" s="42"/>
       <c r="K26" s="42"/>
       <c r="M26" s="42"/>
     </row>
@@ -1939,15 +1967,17 @@
       <c r="H27" t="s">
         <v>74</v>
       </c>
-      <c r="I27"/>
+      <c r="I27" s="42" t="s">
+        <v>96</v>
+      </c>
       <c r="J27" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="K27" s="42" t="s">
         <v>113</v>
       </c>
       <c r="L27" t="s">
-        <v>126</v>
+        <v>154</v>
       </c>
       <c r="M27" s="42" t="s">
         <v>101</v>
@@ -1973,15 +2003,17 @@
       <c r="H28" t="s">
         <v>75</v>
       </c>
-      <c r="I28"/>
+      <c r="I28" s="42" t="s">
+        <v>95</v>
+      </c>
       <c r="J28" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="K28" s="42" t="s">
         <v>114</v>
       </c>
-      <c r="L28" t="s">
-        <v>127</v>
+      <c r="L28" s="42" t="s">
+        <v>153</v>
       </c>
       <c r="M28" s="42" t="s">
         <v>102</v>
@@ -2017,7 +2049,9 @@
       <c r="H30" t="s">
         <v>86</v>
       </c>
-      <c r="I30"/>
+      <c r="I30" t="s">
+        <v>86</v>
+      </c>
       <c r="J30" t="s">
         <v>86</v>
       </c>
@@ -2053,7 +2087,9 @@
       <c r="H31" t="s">
         <v>87</v>
       </c>
-      <c r="I31"/>
+      <c r="I31" t="s">
+        <v>87</v>
+      </c>
       <c r="J31" t="s">
         <v>87</v>
       </c>
@@ -2099,7 +2135,9 @@
       <c r="H33" s="38" t="s">
         <v>88</v>
       </c>
-      <c r="I33" s="38"/>
+      <c r="I33" s="38" t="s">
+        <v>88</v>
+      </c>
       <c r="J33" s="38" t="s">
         <v>88</v>
       </c>
@@ -2133,7 +2171,9 @@
       <c r="H34" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="I34" s="38"/>
+      <c r="I34" s="38" t="s">
+        <v>89</v>
+      </c>
       <c r="J34" s="38" t="s">
         <v>89</v>
       </c>
@@ -2164,7 +2204,9 @@
       <c r="H35" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="I35" s="38"/>
+      <c r="I35" s="38" t="s">
+        <v>90</v>
+      </c>
       <c r="J35" s="38" t="s">
         <v>90</v>
       </c>
@@ -2195,7 +2237,9 @@
       <c r="H36" t="s">
         <v>81</v>
       </c>
-      <c r="I36"/>
+      <c r="I36" t="s">
+        <v>84</v>
+      </c>
       <c r="J36" t="s">
         <v>84</v>
       </c>
@@ -2206,7 +2250,7 @@
         <v>84</v>
       </c>
       <c r="M36" s="42" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -2235,7 +2279,9 @@
       <c r="H38" t="s">
         <v>82</v>
       </c>
-      <c r="I38"/>
+      <c r="I38" t="s">
+        <v>85</v>
+      </c>
       <c r="J38" t="s">
         <v>85</v>
       </c>
@@ -2246,7 +2292,7 @@
         <v>85</v>
       </c>
       <c r="M38" s="42" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="39" spans="1:13">
@@ -2260,7 +2306,9 @@
       <c r="H39" t="s">
         <v>118</v>
       </c>
-      <c r="I39"/>
+      <c r="I39" t="s">
+        <v>117</v>
+      </c>
       <c r="J39" t="s">
         <v>117</v>
       </c>
@@ -2294,7 +2342,9 @@
       <c r="H40" t="s">
         <v>91</v>
       </c>
-      <c r="I40"/>
+      <c r="I40" t="s">
+        <v>44</v>
+      </c>
       <c r="J40" t="s">
         <v>44</v>
       </c>
@@ -2328,7 +2378,9 @@
       <c r="H41" t="s">
         <v>92</v>
       </c>
-      <c r="I41"/>
+      <c r="I41" t="s">
+        <v>45</v>
+      </c>
       <c r="J41" t="s">
         <v>45</v>
       </c>
@@ -2354,7 +2406,9 @@
       </c>
       <c r="E42" s="20"/>
       <c r="H42"/>
-      <c r="I42"/>
+      <c r="I42" s="43" t="s">
+        <v>119</v>
+      </c>
       <c r="J42" s="43" t="s">
         <v>119</v>
       </c>
@@ -2365,7 +2419,7 @@
         <v>119</v>
       </c>
       <c r="M42" s="42" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -2385,7 +2439,9 @@
       <c r="H43" t="s">
         <v>83</v>
       </c>
-      <c r="I43"/>
+      <c r="I43" s="43" t="s">
+        <v>119</v>
+      </c>
       <c r="J43" s="43" t="s">
         <v>119</v>
       </c>
@@ -2409,7 +2465,9 @@
       </c>
       <c r="E44" s="20"/>
       <c r="H44"/>
-      <c r="I44"/>
+      <c r="I44" s="43" t="s">
+        <v>119</v>
+      </c>
       <c r="J44" s="43" t="s">
         <v>119</v>
       </c>
@@ -2420,7 +2478,7 @@
         <v>119</v>
       </c>
       <c r="M44" s="42" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -2481,6 +2539,9 @@
     </row>
     <row r="50" spans="1:12" ht="18.75" thickBot="1">
       <c r="B50" s="2"/>
+      <c r="L50" s="42" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="51" spans="1:12" ht="18.75" thickBot="1">
       <c r="B51" s="40" t="s">
@@ -2530,8 +2591,9 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="J21:J28">
     <sortCondition descending="1" ref="J21:J28"/>
   </sortState>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="B1:E1"/>
+    <mergeCell ref="C2:D2"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2559,7 +2621,7 @@
         <v>93</v>
       </c>
       <c r="D1" s="30" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E1" s="30" t="s">
         <v>93</v>
@@ -2579,7 +2641,7 @@
         <v>78</v>
       </c>
       <c r="E2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2596,7 +2658,7 @@
         <v>79</v>
       </c>
       <c r="E3" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2640,7 +2702,7 @@
         <v>63</v>
       </c>
       <c r="E6" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2807,13 +2869,13 @@
         <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D17" t="s">
         <v>71</v>
       </c>
-      <c r="E17" s="42" t="s">
-        <v>124</v>
+      <c r="E17" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2824,13 +2886,13 @@
         <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D18" t="s">
         <v>72</v>
       </c>
       <c r="E18" t="s">
-        <v>125</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -2851,13 +2913,13 @@
         <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D20" t="s">
         <v>74</v>
       </c>
       <c r="E20" t="s">
-        <v>126</v>
+        <v>155</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="18.75" thickBot="1">
@@ -2868,13 +2930,13 @@
         <v>15</v>
       </c>
       <c r="C21" s="42" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D21" t="s">
         <v>75</v>
       </c>
-      <c r="E21" t="s">
-        <v>127</v>
+      <c r="E21" s="42" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="5" customFormat="1" ht="18.75" thickBot="1">

</xml_diff>

<commit_message>
Added 3.0 HW and updates
Implemented architectural standards for my RPiPico nodes
</commit_message>
<xml_diff>
--- a/Documentation/rp-pico-2-pin-planner-LCCboards.xlsx
+++ b/Documentation/rp-pico-2-pin-planner-LCCboards.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Attic\Documents\Sandboxing\LCC_RPiPico_Turntable\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597FE2EC-6856-4D16-AE35-25CD9EA5C488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46A12F56-7BAD-41FC-98F8-1B4A554CDDA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8475" yWindow="0" windowWidth="40470" windowHeight="20985" xr2:uid="{9994E188-9327-AB46-AF3F-8738237FB097}"/>
+    <workbookView xWindow="8475" yWindow="285" windowWidth="40470" windowHeight="15345" xr2:uid="{9994E188-9327-AB46-AF3F-8738237FB097}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1 (2)" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1 (3)" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="157">
   <si>
     <t>gp0</t>
   </si>
@@ -1284,10 +1285,11 @@
     <col min="5" max="5" width="9.26953125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="2.81640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="20.26953125" hidden="1" customWidth="1"/>
-    <col min="8" max="10" width="20.26953125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="20.26953125" customWidth="1"/>
-    <col min="12" max="12" width="24.26953125" customWidth="1"/>
-    <col min="13" max="13" width="20.08984375" customWidth="1"/>
+    <col min="8" max="9" width="20.26953125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="20.26953125" customWidth="1"/>
+    <col min="11" max="11" width="20.08984375" customWidth="1"/>
+    <col min="12" max="12" width="20.26953125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="24.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="18.75" thickBot="1">
@@ -1300,8 +1302,8 @@
       <c r="C1" s="44"/>
       <c r="D1" s="44"/>
       <c r="E1" s="45"/>
+      <c r="H1" s="31"/>
       <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
@@ -1357,22 +1359,22 @@
         <v>128</v>
       </c>
       <c r="H8" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="I8" s="30" t="s">
+        <v>125</v>
+      </c>
+      <c r="J8" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="K8" s="30" t="s">
+        <v>129</v>
+      </c>
+      <c r="L8" s="30" t="s">
         <v>127</v>
       </c>
-      <c r="I8" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="J8" s="30" t="s">
-        <v>125</v>
-      </c>
-      <c r="K8" s="30" t="s">
-        <v>94</v>
-      </c>
-      <c r="L8" s="30" t="s">
+      <c r="M8" s="30" t="s">
         <v>93</v>
-      </c>
-      <c r="M8" s="30" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1394,23 +1396,23 @@
       <c r="G9" t="s">
         <v>60</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="I9" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="J9" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="K9" t="s">
+        <v>86</v>
+      </c>
+      <c r="L9" t="s">
         <v>78</v>
       </c>
-      <c r="I9" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="J9" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="K9" s="42" t="s">
-        <v>95</v>
-      </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>142</v>
-      </c>
-      <c r="M9" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1432,23 +1434,23 @@
       <c r="G10" t="s">
         <v>61</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="I10" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="J10" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="K10" t="s">
+        <v>87</v>
+      </c>
+      <c r="L10" t="s">
         <v>79</v>
       </c>
-      <c r="I10" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="J10" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="K10" s="42" t="s">
-        <v>96</v>
-      </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>143</v>
-      </c>
-      <c r="M10" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1461,8 +1463,8 @@
       <c r="E11" s="20"/>
       <c r="H11"/>
       <c r="I11"/>
-      <c r="J11"/>
-      <c r="K11" s="42"/>
+      <c r="J11" s="42"/>
+      <c r="L11"/>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="7">
@@ -1482,22 +1484,22 @@
         <v>62</v>
       </c>
       <c r="H12" t="s">
-        <v>80</v>
+        <v>130</v>
       </c>
       <c r="I12" t="s">
         <v>130</v>
       </c>
-      <c r="J12" t="s">
-        <v>130</v>
-      </c>
-      <c r="K12" s="42" t="s">
+      <c r="J12" s="42" t="s">
         <v>97</v>
+      </c>
+      <c r="K12" s="38" t="s">
+        <v>88</v>
       </c>
       <c r="L12" t="s">
         <v>80</v>
       </c>
-      <c r="M12" s="38" t="s">
-        <v>88</v>
+      <c r="M12" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1518,22 +1520,22 @@
         <v>63</v>
       </c>
       <c r="H13" t="s">
-        <v>63</v>
+        <v>131</v>
       </c>
       <c r="I13" t="s">
         <v>131</v>
       </c>
-      <c r="J13" t="s">
-        <v>131</v>
-      </c>
-      <c r="K13" s="42" t="s">
+      <c r="J13" s="42" t="s">
         <v>98</v>
       </c>
+      <c r="K13" s="38" t="s">
+        <v>89</v>
+      </c>
       <c r="L13" t="s">
+        <v>63</v>
+      </c>
+      <c r="M13" t="s">
         <v>144</v>
-      </c>
-      <c r="M13" s="38" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -1555,23 +1557,23 @@
       <c r="G14" t="s">
         <v>64</v>
       </c>
-      <c r="H14" t="s">
-        <v>64</v>
+      <c r="H14" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="K14" s="42" t="s">
+      <c r="J14" s="42" t="s">
         <v>115</v>
       </c>
-      <c r="L14" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="M14" s="38" t="s">
+      <c r="K14" s="38" t="s">
         <v>90</v>
+      </c>
+      <c r="L14" t="s">
+        <v>64</v>
+      </c>
+      <c r="M14" s="43" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -1593,20 +1595,20 @@
       <c r="G15" t="s">
         <v>65</v>
       </c>
-      <c r="H15" t="s">
-        <v>65</v>
+      <c r="H15" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J15" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="K15" s="42" t="s">
+      <c r="J15" s="42" t="s">
         <v>116</v>
       </c>
-      <c r="L15" s="43" t="s">
-        <v>119</v>
+      <c r="K15" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="L15" t="s">
+        <v>65</v>
       </c>
       <c r="M15" s="43" t="s">
         <v>119</v>
@@ -1622,8 +1624,8 @@
       <c r="E16" s="20"/>
       <c r="H16"/>
       <c r="I16"/>
-      <c r="J16"/>
-      <c r="K16" s="42"/>
+      <c r="J16" s="42"/>
+      <c r="L16"/>
     </row>
     <row r="17" spans="1:13">
       <c r="A17" s="7">
@@ -1643,22 +1645,22 @@
         <v>73</v>
       </c>
       <c r="H17" t="s">
-        <v>73</v>
+        <v>132</v>
       </c>
       <c r="I17" t="s">
         <v>132</v>
       </c>
-      <c r="J17" t="s">
-        <v>132</v>
-      </c>
-      <c r="K17" s="42" t="s">
+      <c r="J17" s="42" t="s">
         <v>101</v>
       </c>
+      <c r="K17" t="s">
+        <v>44</v>
+      </c>
       <c r="L17" t="s">
+        <v>73</v>
+      </c>
+      <c r="M17" t="s">
         <v>74</v>
-      </c>
-      <c r="M17" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -1679,22 +1681,22 @@
         <v>66</v>
       </c>
       <c r="H18" t="s">
-        <v>66</v>
+        <v>133</v>
       </c>
       <c r="I18" t="s">
         <v>133</v>
       </c>
-      <c r="J18" t="s">
-        <v>133</v>
-      </c>
-      <c r="K18" s="42" t="s">
+      <c r="J18" s="42" t="s">
         <v>102</v>
       </c>
+      <c r="K18" t="s">
+        <v>45</v>
+      </c>
       <c r="L18" t="s">
+        <v>66</v>
+      </c>
+      <c r="M18" t="s">
         <v>75</v>
-      </c>
-      <c r="M18" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -1716,23 +1718,23 @@
       <c r="G19" t="s">
         <v>67</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" s="42" t="s">
+        <v>102</v>
+      </c>
+      <c r="I19" t="s">
+        <v>134</v>
+      </c>
+      <c r="J19" s="42" t="s">
+        <v>103</v>
+      </c>
+      <c r="K19" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="L19" t="s">
         <v>67</v>
       </c>
-      <c r="I19" s="42" t="s">
-        <v>102</v>
-      </c>
-      <c r="J19" t="s">
-        <v>134</v>
-      </c>
-      <c r="K19" s="42" t="s">
-        <v>103</v>
-      </c>
-      <c r="L19" t="s">
+      <c r="M19" t="s">
         <v>120</v>
-      </c>
-      <c r="M19" s="42" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -1754,23 +1756,23 @@
       <c r="G20" t="s">
         <v>68</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="42" t="s">
+        <v>101</v>
+      </c>
+      <c r="I20" t="s">
+        <v>135</v>
+      </c>
+      <c r="J20" s="42" t="s">
+        <v>104</v>
+      </c>
+      <c r="K20" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="L20" t="s">
         <v>68</v>
       </c>
-      <c r="I20" s="42" t="s">
-        <v>101</v>
-      </c>
-      <c r="J20" t="s">
-        <v>135</v>
-      </c>
-      <c r="K20" s="42" t="s">
-        <v>104</v>
-      </c>
-      <c r="L20" t="s">
+      <c r="M20" t="s">
         <v>121</v>
-      </c>
-      <c r="M20" s="42" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -1781,10 +1783,10 @@
         <v>26</v>
       </c>
       <c r="E21" s="20"/>
-      <c r="H21"/>
-      <c r="I21" s="42"/>
+      <c r="H21" s="42"/>
+      <c r="J21" s="42"/>
       <c r="K21" s="42"/>
-      <c r="M21" s="42"/>
+      <c r="L21"/>
     </row>
     <row r="22" spans="1:13">
       <c r="A22" s="7">
@@ -1803,23 +1805,23 @@
       <c r="G22" t="s">
         <v>69</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H22" s="42" t="s">
+        <v>146</v>
+      </c>
+      <c r="I22" t="s">
+        <v>141</v>
+      </c>
+      <c r="J22" s="42" t="s">
+        <v>105</v>
+      </c>
+      <c r="K22" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="L22" t="s">
         <v>69</v>
       </c>
-      <c r="I22" s="42" t="s">
-        <v>146</v>
-      </c>
-      <c r="J22" t="s">
-        <v>141</v>
-      </c>
-      <c r="K22" s="42" t="s">
-        <v>105</v>
-      </c>
-      <c r="L22" t="s">
+      <c r="M22" t="s">
         <v>122</v>
-      </c>
-      <c r="M22" s="42" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -1839,23 +1841,23 @@
       <c r="G23" t="s">
         <v>70</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H23" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="I23" t="s">
+        <v>140</v>
+      </c>
+      <c r="J23" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="K23" s="42" t="s">
+        <v>98</v>
+      </c>
+      <c r="L23" t="s">
         <v>70</v>
       </c>
-      <c r="I23" s="42" t="s">
-        <v>145</v>
-      </c>
-      <c r="J23" t="s">
-        <v>140</v>
-      </c>
-      <c r="K23" s="42" t="s">
-        <v>106</v>
-      </c>
-      <c r="L23" t="s">
+      <c r="M23" t="s">
         <v>123</v>
-      </c>
-      <c r="M23" s="42" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -1877,23 +1879,23 @@
       <c r="G24" t="s">
         <v>71</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H24" s="42" t="s">
+        <v>98</v>
+      </c>
+      <c r="I24" t="s">
+        <v>139</v>
+      </c>
+      <c r="J24" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="K24" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="L24" t="s">
         <v>71</v>
       </c>
-      <c r="I24" s="42" t="s">
-        <v>98</v>
-      </c>
-      <c r="J24" t="s">
-        <v>139</v>
-      </c>
-      <c r="K24" s="42" t="s">
-        <v>109</v>
-      </c>
-      <c r="L24" t="s">
+      <c r="M24" t="s">
         <v>151</v>
-      </c>
-      <c r="M24" s="42" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -1915,23 +1917,23 @@
       <c r="G25" t="s">
         <v>72</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H25" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="I25" t="s">
+        <v>138</v>
+      </c>
+      <c r="J25" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="K25" s="42" t="s">
+        <v>146</v>
+      </c>
+      <c r="L25" t="s">
         <v>72</v>
       </c>
-      <c r="I25" s="42" t="s">
-        <v>97</v>
-      </c>
-      <c r="J25" t="s">
-        <v>138</v>
-      </c>
-      <c r="K25" s="42" t="s">
-        <v>112</v>
-      </c>
-      <c r="L25" t="s">
+      <c r="M25" t="s">
         <v>152</v>
-      </c>
-      <c r="M25" s="42" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -1942,10 +1944,10 @@
         <v>26</v>
       </c>
       <c r="E26" s="20"/>
-      <c r="H26"/>
-      <c r="I26" s="42"/>
+      <c r="H26" s="42"/>
+      <c r="J26" s="42"/>
       <c r="K26" s="42"/>
-      <c r="M26" s="42"/>
+      <c r="L26"/>
     </row>
     <row r="27" spans="1:13">
       <c r="A27" s="7">
@@ -1964,23 +1966,23 @@
       <c r="G27" t="s">
         <v>74</v>
       </c>
-      <c r="H27" t="s">
+      <c r="H27" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="I27" t="s">
+        <v>137</v>
+      </c>
+      <c r="J27" s="42" t="s">
+        <v>113</v>
+      </c>
+      <c r="K27" s="42" t="s">
+        <v>101</v>
+      </c>
+      <c r="L27" t="s">
         <v>74</v>
       </c>
-      <c r="I27" s="42" t="s">
-        <v>96</v>
-      </c>
-      <c r="J27" t="s">
-        <v>137</v>
-      </c>
-      <c r="K27" s="42" t="s">
-        <v>113</v>
-      </c>
-      <c r="L27" t="s">
+      <c r="M27" t="s">
         <v>154</v>
-      </c>
-      <c r="M27" s="42" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="18.75" thickBot="1">
@@ -2000,23 +2002,23 @@
       <c r="G28" t="s">
         <v>75</v>
       </c>
-      <c r="H28" t="s">
+      <c r="H28" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="I28" t="s">
+        <v>136</v>
+      </c>
+      <c r="J28" s="42" t="s">
+        <v>114</v>
+      </c>
+      <c r="K28" s="42" t="s">
+        <v>102</v>
+      </c>
+      <c r="L28" t="s">
         <v>75</v>
       </c>
-      <c r="I28" s="42" t="s">
-        <v>95</v>
-      </c>
-      <c r="J28" t="s">
-        <v>136</v>
-      </c>
-      <c r="K28" s="42" t="s">
-        <v>114</v>
-      </c>
-      <c r="L28" s="42" t="s">
+      <c r="M28" s="42" t="s">
         <v>153</v>
-      </c>
-      <c r="M28" s="42" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:13" s="5" customFormat="1" ht="18.75" thickBot="1">
@@ -2035,7 +2037,7 @@
         <v>25</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D30" s="17" t="s">
         <v>42</v>
@@ -2055,14 +2057,14 @@
       <c r="J30" t="s">
         <v>86</v>
       </c>
-      <c r="K30" t="s">
-        <v>86</v>
+      <c r="K30" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="L30" t="s">
         <v>86</v>
       </c>
-      <c r="M30" s="1" t="s">
-        <v>42</v>
+      <c r="M30" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -2073,7 +2075,7 @@
         <v>24</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D31" s="34" t="s">
         <v>43</v>
@@ -2093,14 +2095,14 @@
       <c r="J31" t="s">
         <v>87</v>
       </c>
-      <c r="K31" t="s">
-        <v>87</v>
+      <c r="K31" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="L31" t="s">
         <v>87</v>
       </c>
-      <c r="M31" s="1" t="s">
-        <v>43</v>
+      <c r="M31" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -2113,7 +2115,7 @@
       <c r="E32" s="20"/>
       <c r="H32"/>
       <c r="I32"/>
-      <c r="J32"/>
+      <c r="L32"/>
     </row>
     <row r="33" spans="1:13">
       <c r="A33" s="1">
@@ -2123,7 +2125,7 @@
         <v>23</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D33" s="34" t="s">
         <v>44</v>
@@ -2141,14 +2143,14 @@
       <c r="J33" s="38" t="s">
         <v>88</v>
       </c>
-      <c r="K33" s="38" t="s">
-        <v>88</v>
+      <c r="K33" s="42" t="s">
+        <v>103</v>
       </c>
       <c r="L33" s="38" t="s">
         <v>88</v>
       </c>
-      <c r="M33" s="42" t="s">
-        <v>103</v>
+      <c r="M33" s="38" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -2159,7 +2161,7 @@
         <v>22</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D34" s="34" t="s">
         <v>45</v>
@@ -2177,14 +2179,14 @@
       <c r="J34" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="K34" s="38" t="s">
-        <v>89</v>
+      <c r="K34" s="42" t="s">
+        <v>104</v>
       </c>
       <c r="L34" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="M34" s="42" t="s">
-        <v>104</v>
+      <c r="M34" s="38" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -2210,14 +2212,14 @@
       <c r="J35" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="K35" s="38" t="s">
-        <v>90</v>
+      <c r="K35" s="42" t="s">
+        <v>105</v>
       </c>
       <c r="L35" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="M35" s="42" t="s">
-        <v>105</v>
+      <c r="M35" s="38" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -2235,7 +2237,7 @@
         <v>81</v>
       </c>
       <c r="H36" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="I36" t="s">
         <v>84</v>
@@ -2243,14 +2245,14 @@
       <c r="J36" t="s">
         <v>84</v>
       </c>
-      <c r="K36" t="s">
+      <c r="K36" s="42" t="s">
+        <v>147</v>
+      </c>
+      <c r="L36" t="s">
+        <v>81</v>
+      </c>
+      <c r="M36" t="s">
         <v>84</v>
-      </c>
-      <c r="L36" t="s">
-        <v>84</v>
-      </c>
-      <c r="M36" s="42" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -2263,7 +2265,7 @@
       <c r="E37" s="20"/>
       <c r="H37"/>
       <c r="I37"/>
-      <c r="J37"/>
+      <c r="L37"/>
     </row>
     <row r="38" spans="1:13">
       <c r="A38" s="1">
@@ -2277,7 +2279,7 @@
         <v>82</v>
       </c>
       <c r="H38" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I38" t="s">
         <v>85</v>
@@ -2285,14 +2287,14 @@
       <c r="J38" t="s">
         <v>85</v>
       </c>
-      <c r="K38" t="s">
+      <c r="K38" s="42" t="s">
+        <v>148</v>
+      </c>
+      <c r="L38" t="s">
+        <v>82</v>
+      </c>
+      <c r="M38" t="s">
         <v>85</v>
-      </c>
-      <c r="L38" t="s">
-        <v>85</v>
-      </c>
-      <c r="M38" s="42" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="39" spans="1:13">
@@ -2304,7 +2306,7 @@
       </c>
       <c r="E39" s="20"/>
       <c r="H39" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I39" t="s">
         <v>117</v>
@@ -2316,7 +2318,7 @@
         <v>117</v>
       </c>
       <c r="L39" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="M39" t="s">
         <v>117</v>
@@ -2340,7 +2342,7 @@
         <v>44</v>
       </c>
       <c r="H40" t="s">
-        <v>91</v>
+        <v>44</v>
       </c>
       <c r="I40" t="s">
         <v>44</v>
@@ -2348,14 +2350,14 @@
       <c r="J40" t="s">
         <v>44</v>
       </c>
-      <c r="K40" t="s">
+      <c r="K40" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="L40" t="s">
+        <v>91</v>
+      </c>
+      <c r="M40" t="s">
         <v>44</v>
-      </c>
-      <c r="L40" t="s">
-        <v>44</v>
-      </c>
-      <c r="M40" s="42" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="41" spans="1:13">
@@ -2376,7 +2378,7 @@
         <v>45</v>
       </c>
       <c r="H41" t="s">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="I41" t="s">
         <v>45</v>
@@ -2384,14 +2386,14 @@
       <c r="J41" t="s">
         <v>45</v>
       </c>
-      <c r="K41" t="s">
+      <c r="K41" s="42" t="s">
+        <v>113</v>
+      </c>
+      <c r="L41" t="s">
+        <v>92</v>
+      </c>
+      <c r="M41" t="s">
         <v>45</v>
-      </c>
-      <c r="L41" t="s">
-        <v>45</v>
-      </c>
-      <c r="M41" s="42" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="42" spans="1:13">
@@ -2405,21 +2407,21 @@
         <v>53</v>
       </c>
       <c r="E42" s="20"/>
-      <c r="H42"/>
+      <c r="H42" s="43" t="s">
+        <v>119</v>
+      </c>
       <c r="I42" s="43" t="s">
         <v>119</v>
       </c>
       <c r="J42" s="43" t="s">
         <v>119</v>
       </c>
-      <c r="K42" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="L42" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="M42" s="42" t="s">
+      <c r="K42" s="42" t="s">
         <v>149</v>
+      </c>
+      <c r="L42"/>
+      <c r="M42" s="43" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -2436,23 +2438,23 @@
       <c r="G43" t="s">
         <v>83</v>
       </c>
-      <c r="H43" t="s">
+      <c r="H43" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="I43" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="J43" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="K43" s="42" t="s">
+        <v>114</v>
+      </c>
+      <c r="L43" t="s">
         <v>83</v>
       </c>
-      <c r="I43" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="J43" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="K43" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="L43" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="M43" s="42" t="s">
-        <v>114</v>
+      <c r="M43" s="43" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -2464,21 +2466,21 @@
         <v>41</v>
       </c>
       <c r="E44" s="20"/>
-      <c r="H44"/>
+      <c r="H44" s="43" t="s">
+        <v>119</v>
+      </c>
       <c r="I44" s="43" t="s">
         <v>119</v>
       </c>
       <c r="J44" s="43" t="s">
         <v>119</v>
       </c>
-      <c r="K44" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="L44" s="43" t="s">
-        <v>119</v>
-      </c>
-      <c r="M44" s="42" t="s">
+      <c r="K44" s="42" t="s">
         <v>150</v>
+      </c>
+      <c r="L44"/>
+      <c r="M44" s="43" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -2491,7 +2493,7 @@
       <c r="E45" s="20"/>
       <c r="H45"/>
       <c r="I45"/>
-      <c r="J45"/>
+      <c r="L45"/>
     </row>
     <row r="46" spans="1:13">
       <c r="A46" s="1">
@@ -2503,7 +2505,7 @@
       <c r="E46" s="20"/>
       <c r="H46"/>
       <c r="I46"/>
-      <c r="J46"/>
+      <c r="L46"/>
     </row>
     <row r="47" spans="1:13">
       <c r="A47" s="1">
@@ -2515,7 +2517,7 @@
       <c r="E47" s="20"/>
       <c r="H47"/>
       <c r="I47"/>
-      <c r="J47"/>
+      <c r="L47"/>
     </row>
     <row r="48" spans="1:13">
       <c r="A48" s="1">
@@ -2526,7 +2528,7 @@
       </c>
       <c r="E48" s="20"/>
     </row>
-    <row r="49" spans="1:12" ht="18.75" thickBot="1">
+    <row r="49" spans="1:13" ht="18.75" thickBot="1">
       <c r="A49" s="1">
         <v>40</v>
       </c>
@@ -2537,59 +2539,59 @@
       <c r="D49" s="24"/>
       <c r="E49" s="23"/>
     </row>
-    <row r="50" spans="1:12" ht="18.75" thickBot="1">
+    <row r="50" spans="1:13" ht="18.75" thickBot="1">
       <c r="B50" s="2"/>
-      <c r="L50" s="42" t="s">
+      <c r="M50" s="42" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="51" spans="1:12" ht="18.75" thickBot="1">
+    <row r="51" spans="1:13" ht="18.75" thickBot="1">
       <c r="B51" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="K51" t="s">
+      <c r="J51" t="s">
         <v>99</v>
       </c>
-      <c r="L51" t="s">
+      <c r="M51" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="52" spans="1:12" ht="18.75" thickBot="1">
+    <row r="52" spans="1:13" ht="18.75" thickBot="1">
       <c r="B52" s="41" t="s">
         <v>110</v>
       </c>
-      <c r="K52" t="s">
+      <c r="J52" t="s">
         <v>100</v>
       </c>
-      <c r="L52" t="s">
+      <c r="M52" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:12" ht="18.75" thickBot="1">
+    <row r="53" spans="1:13" ht="18.75" thickBot="1">
       <c r="B53" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="K53" t="s">
+      <c r="J53" t="s">
         <v>107</v>
       </c>
-      <c r="L53" t="s">
+      <c r="M53" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="54" spans="1:12" ht="18.75" thickBot="1">
+    <row r="54" spans="1:13" ht="18.75" thickBot="1">
       <c r="B54" s="41" t="s">
         <v>111</v>
       </c>
-      <c r="K54" t="s">
+      <c r="J54" t="s">
         <v>108</v>
       </c>
-      <c r="L54" t="s">
+      <c r="M54" t="s">
         <v>108</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="J21:J28">
-    <sortCondition descending="1" ref="J21:J28"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="I21:I28">
+    <sortCondition descending="1" ref="I21:I28"/>
   </sortState>
   <mergeCells count="2">
     <mergeCell ref="B1:E1"/>
@@ -3224,4 +3226,732 @@
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="53" orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22879F06-826D-4665-AFBE-58D1FA19CBEA}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr defaultColWidth="11.08984375" defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="5.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.36328125" customWidth="1"/>
+    <col min="5" max="5" width="26.6328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="20.26953125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="24.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="18.75" thickBot="1">
+      <c r="C1" s="30" t="s">
+        <v>129</v>
+      </c>
+      <c r="E1" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="F1" s="30" t="s">
+        <v>125</v>
+      </c>
+      <c r="G1" s="30" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E2" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="F2" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="G2" s="42" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="7">
+        <v>2</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="F3" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="G3" s="42" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="7">
+        <v>3</v>
+      </c>
+      <c r="B4" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4"/>
+      <c r="F4"/>
+      <c r="G4" s="42"/>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="7">
+        <v>4</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="E5" t="s">
+        <v>130</v>
+      </c>
+      <c r="F5" t="s">
+        <v>130</v>
+      </c>
+      <c r="G5" s="42" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="7">
+        <v>5</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="E6" t="s">
+        <v>131</v>
+      </c>
+      <c r="F6" t="s">
+        <v>131</v>
+      </c>
+      <c r="G6" s="42" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" s="42" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="7">
+        <v>7</v>
+      </c>
+      <c r="B8" s="32" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="42" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="7">
+        <v>8</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9" s="42"/>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="7">
+        <v>9</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" t="s">
+        <v>132</v>
+      </c>
+      <c r="F10" t="s">
+        <v>132</v>
+      </c>
+      <c r="G10" s="42" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="7">
+        <v>10</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" t="s">
+        <v>133</v>
+      </c>
+      <c r="F11" t="s">
+        <v>133</v>
+      </c>
+      <c r="G11" s="42" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="7">
+        <v>11</v>
+      </c>
+      <c r="B12" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="E12" s="42" t="s">
+        <v>102</v>
+      </c>
+      <c r="F12" t="s">
+        <v>134</v>
+      </c>
+      <c r="G12" s="42" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="7">
+        <v>12</v>
+      </c>
+      <c r="B13" s="32" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="E13" s="42" t="s">
+        <v>101</v>
+      </c>
+      <c r="F13" t="s">
+        <v>135</v>
+      </c>
+      <c r="G13" s="42" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="7">
+        <v>13</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="G14" s="42"/>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="7">
+        <v>14</v>
+      </c>
+      <c r="B15" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="E15" s="42" t="s">
+        <v>146</v>
+      </c>
+      <c r="F15" t="s">
+        <v>141</v>
+      </c>
+      <c r="G15" s="42" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="7">
+        <v>15</v>
+      </c>
+      <c r="B16" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="42" t="s">
+        <v>98</v>
+      </c>
+      <c r="E16" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="F16" t="s">
+        <v>140</v>
+      </c>
+      <c r="G16" s="42" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="7">
+        <v>16</v>
+      </c>
+      <c r="B17" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="E17" s="42" t="s">
+        <v>98</v>
+      </c>
+      <c r="F17" t="s">
+        <v>139</v>
+      </c>
+      <c r="G17" s="42" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="7">
+        <v>17</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="42" t="s">
+        <v>146</v>
+      </c>
+      <c r="E18" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="F18" t="s">
+        <v>138</v>
+      </c>
+      <c r="G18" s="42" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="7">
+        <v>18</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="G19" s="42"/>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="7">
+        <v>19</v>
+      </c>
+      <c r="B20" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="42" t="s">
+        <v>101</v>
+      </c>
+      <c r="E20" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="F20" t="s">
+        <v>137</v>
+      </c>
+      <c r="G20" s="42" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="18.75" thickBot="1">
+      <c r="A21" s="8">
+        <v>20</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="42" t="s">
+        <v>102</v>
+      </c>
+      <c r="E21" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="F21" t="s">
+        <v>136</v>
+      </c>
+      <c r="G21" s="42" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" s="5" customFormat="1" ht="18.75" thickBot="1">
+      <c r="A22" s="3"/>
+      <c r="B22" s="4"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="1">
+        <v>21</v>
+      </c>
+      <c r="B23" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E23" t="s">
+        <v>86</v>
+      </c>
+      <c r="F23" t="s">
+        <v>86</v>
+      </c>
+      <c r="G23" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="1">
+        <v>22</v>
+      </c>
+      <c r="B24" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E24" t="s">
+        <v>87</v>
+      </c>
+      <c r="F24" t="s">
+        <v>87</v>
+      </c>
+      <c r="G24" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="1">
+        <v>23</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25"/>
+      <c r="F25"/>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="1">
+        <v>24</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="C26" s="42" t="s">
+        <v>103</v>
+      </c>
+      <c r="E26" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="F26" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="G26" s="38" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="1">
+        <v>25</v>
+      </c>
+      <c r="B27" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27" s="42" t="s">
+        <v>104</v>
+      </c>
+      <c r="E27" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="F27" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="G27" s="38" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="1">
+        <v>26</v>
+      </c>
+      <c r="B28" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" s="42" t="s">
+        <v>105</v>
+      </c>
+      <c r="E28" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="F28" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="G28" s="38" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="1">
+        <v>27</v>
+      </c>
+      <c r="B29" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="42" t="s">
+        <v>147</v>
+      </c>
+      <c r="E29" t="s">
+        <v>84</v>
+      </c>
+      <c r="F29" t="s">
+        <v>84</v>
+      </c>
+      <c r="G29" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="1">
+        <v>28</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30"/>
+      <c r="F30"/>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="1">
+        <v>29</v>
+      </c>
+      <c r="B31" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" s="42" t="s">
+        <v>148</v>
+      </c>
+      <c r="E31" t="s">
+        <v>85</v>
+      </c>
+      <c r="F31" t="s">
+        <v>85</v>
+      </c>
+      <c r="G31" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="1">
+        <v>30</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" t="s">
+        <v>117</v>
+      </c>
+      <c r="E32" t="s">
+        <v>117</v>
+      </c>
+      <c r="F32" t="s">
+        <v>117</v>
+      </c>
+      <c r="G32" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="1">
+        <v>31</v>
+      </c>
+      <c r="B33" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="E33" t="s">
+        <v>44</v>
+      </c>
+      <c r="F33" t="s">
+        <v>44</v>
+      </c>
+      <c r="G33" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="1">
+        <v>32</v>
+      </c>
+      <c r="B34" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" s="42" t="s">
+        <v>113</v>
+      </c>
+      <c r="E34" t="s">
+        <v>45</v>
+      </c>
+      <c r="F34" t="s">
+        <v>45</v>
+      </c>
+      <c r="G34" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="1">
+        <v>33</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C35" s="42" t="s">
+        <v>149</v>
+      </c>
+      <c r="E35" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="F35" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="G35" s="43" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="1">
+        <v>34</v>
+      </c>
+      <c r="B36" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="42" t="s">
+        <v>114</v>
+      </c>
+      <c r="E36" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="F36" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="G36" s="43" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="1">
+        <v>35</v>
+      </c>
+      <c r="B37" s="7"/>
+      <c r="C37" s="42" t="s">
+        <v>150</v>
+      </c>
+      <c r="E37" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="F37" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="G37" s="43" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="1">
+        <v>36</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="E38"/>
+      <c r="F38"/>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="1">
+        <v>37</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="E39"/>
+      <c r="F39"/>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="1">
+        <v>38</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E40"/>
+      <c r="F40"/>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="1">
+        <v>39</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="18.75" thickBot="1">
+      <c r="A42" s="1">
+        <v>40</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="53" orientation="landscape" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>